<commit_message>
chore(meshika): refresh live outputs (EPPA re-run + renamed merged page)
Runtime outputs from the proven EPPA weekly run + merged republish under the clearer name:
eppa dashboard/workbook/data.json (48 campaigns, anchor 2026-08-13) and the merged page.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/development/abiraj_mini_aios_workbench/projects/PRJ-2026-013_ebay-ppc-product-pause-automation/evidence/final_outputs/REQ-15_ebay-ppc-product-pause-automation/REQ-15-D01_eppa_pause_log.xlsx
+++ b/development/abiraj_mini_aios_workbench/projects/PRJ-2026-013_ebay-ppc-product-pause-automation/evidence/final_outputs/REQ-15_ebay-ppc-product-pause-automation/REQ-15-D01_eppa_pause_log.xlsx
@@ -543,7 +543,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>30D 12 Jul - 10 Aug 2026  ·  14D 28 Jul - 10 Aug 2026  ·  7D 4-10 Aug 2026   (each window ends on 10 Aug 2026 and includes it)</t>
+          <t>30D 15 Jul - 13 Aug 2026  ·  14D 31 Jul - 13 Aug 2026  ·  7D 7-13 Aug 2026   (each window ends on 13 Aug 2026 and includes it)</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9">
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10">
@@ -603,7 +603,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -623,7 +623,7 @@
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13">
@@ -633,7 +633,7 @@
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">
@@ -643,7 +643,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="16">
@@ -663,7 +663,7 @@
         </is>
       </c>
       <c r="B16" s="4" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="17">
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>714.5599999999999</v>
+        <v>902.38</v>
       </c>
     </row>
     <row r="18">
@@ -683,7 +683,7 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>2905.19</v>
+        <v>2896.02</v>
       </c>
     </row>
     <row r="19">
@@ -693,7 +693,7 @@
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>1177</v>
+        <v>1149</v>
       </c>
     </row>
     <row r="20">
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B20" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="21">
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B21" s="4" t="n">
-        <v>47</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -904,25 +904,25 @@
         </is>
       </c>
       <c r="K2" s="7" t="n">
-        <v>24.9</v>
+        <v>29.3</v>
       </c>
       <c r="L2" s="7" t="n">
-        <v>57</v>
+        <v>37.9</v>
       </c>
       <c r="M2" s="7" t="n">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="N2" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="P2" s="9" t="n">
-        <v>53.16</v>
+        <v>54.31</v>
       </c>
       <c r="Q2" s="9" t="n">
-        <v>127.3</v>
+        <v>126.29</v>
       </c>
       <c r="R2" s="7" t="inlineStr">
         <is>
@@ -944,17 +944,17 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>JD | PH | Pendant Light Fitting  | Tharshana | Manual</t>
+          <t>JD | stock clearance products | Smart</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>160677049012</t>
+          <t>28863477012</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>Manual</t>
+          <t>Smart</t>
         </is>
       </c>
       <c r="D3" s="7" t="inlineStr">
@@ -963,7 +963,7 @@
         </is>
       </c>
       <c r="E3" s="7" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="F3" s="7" t="n">
         <v>1</v>
@@ -972,7 +972,7 @@
         <v>0</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
@@ -985,25 +985,25 @@
         </is>
       </c>
       <c r="K3" s="7" t="n">
-        <v>21.4</v>
+        <v>14.8</v>
       </c>
       <c r="L3" s="7" t="n">
-        <v>39.2</v>
+        <v>15</v>
       </c>
       <c r="M3" s="7" t="n">
-        <v>31</v>
+        <v>52</v>
       </c>
       <c r="N3" s="7" t="n">
-        <v>22</v>
+        <v>39</v>
       </c>
       <c r="O3" s="7" t="n">
-        <v>236</v>
+        <v>344</v>
       </c>
       <c r="P3" s="9" t="n">
-        <v>42.91</v>
+        <v>66.81999999999999</v>
       </c>
       <c r="Q3" s="9" t="n">
-        <v>96.37</v>
+        <v>101.89</v>
       </c>
       <c r="R3" s="7" t="inlineStr">
         <is>
@@ -1012,7 +1012,7 @@
       </c>
       <c r="S3" s="10" t="inlineStr">
         <is>
-          <t>1 of the 40 listings this campaign advertises is out of stock (0 units). Ads are paused so spend does not keep running on items that cannot be bought.</t>
+          <t>1 of the 30 listings this campaign advertises is out of stock (0 units). Ads are paused so spend does not keep running on items that cannot be bought.</t>
         </is>
       </c>
       <c r="T3" s="7" t="inlineStr">
@@ -1025,17 +1025,17 @@
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>JD | stock clearance products | Smart</t>
+          <t>JD | PH | Pendant Light Fitting  | Tharshana | Manual</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>28863477012</t>
+          <t>160677049012</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>Smart</t>
+          <t>Manual</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
@@ -1044,7 +1044,7 @@
         </is>
       </c>
       <c r="E4" s="7" t="n">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="F4" s="7" t="n">
         <v>1</v>
@@ -1066,25 +1066,25 @@
         </is>
       </c>
       <c r="K4" s="7" t="n">
-        <v>14.2</v>
+        <v>22.3</v>
       </c>
       <c r="L4" s="7" t="n">
-        <v>34.6</v>
+        <v>39.5</v>
       </c>
       <c r="M4" s="7" t="n">
-        <v>43</v>
+        <v>30</v>
       </c>
       <c r="N4" s="7" t="n">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="O4" s="7" t="n">
-        <v>300</v>
+        <v>231</v>
       </c>
       <c r="P4" s="9" t="n">
-        <v>58.49</v>
+        <v>42.98</v>
       </c>
       <c r="Q4" s="9" t="n">
-        <v>94.78</v>
+        <v>96.84999999999999</v>
       </c>
       <c r="R4" s="7" t="inlineStr">
         <is>
@@ -1093,7 +1093,7 @@
       </c>
       <c r="S4" s="10" t="inlineStr">
         <is>
-          <t>1 of the 30 listings this campaign advertises is out of stock (0 units). Ads are paused so spend does not keep running on items that cannot be bought.</t>
+          <t>1 of the 36 listings this campaign advertises is out of stock (0 units). Ads are paused so spend does not keep running on items that cannot be bought.</t>
         </is>
       </c>
       <c r="T4" s="7" t="inlineStr">
@@ -1147,25 +1147,23 @@
         </is>
       </c>
       <c r="K5" s="7" t="n">
-        <v>23.1</v>
-      </c>
-      <c r="L5" s="7" t="n">
-        <v>18.8</v>
-      </c>
+        <v>23.2</v>
+      </c>
+      <c r="L5" s="7" t="n"/>
       <c r="M5" s="7" t="n">
         <v>10</v>
       </c>
       <c r="N5" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O5" s="7" t="n">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="P5" s="9" t="n">
-        <v>43.48</v>
+        <v>42.07</v>
       </c>
       <c r="Q5" s="9" t="n">
-        <v>93.77</v>
+        <v>94.16</v>
       </c>
       <c r="R5" s="7" t="inlineStr">
         <is>
@@ -1187,12 +1185,12 @@
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>JD | Ceiling Lights | Manual</t>
+          <t>JD | MH | Flush Light &amp; Lamp Shade | Shanthini | Manual</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>163193938012</t>
+          <t>159902435012</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
@@ -1206,7 +1204,7 @@
         </is>
       </c>
       <c r="E6" s="7" t="n">
-        <v>75</v>
+        <v>38</v>
       </c>
       <c r="F6" s="7" t="n">
         <v>1</v>
@@ -1215,38 +1213,38 @@
         <v>0</v>
       </c>
       <c r="H6" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="J6" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K6" s="7" t="n">
+        <v>42.3</v>
+      </c>
+      <c r="L6" s="7" t="n">
+        <v>176.4</v>
+      </c>
+      <c r="M6" s="7" t="n">
+        <v>17</v>
+      </c>
+      <c r="N6" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="I6" s="8" t="inlineStr">
-        <is>
-          <t>Stock</t>
-        </is>
-      </c>
-      <c r="J6" s="7" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="K6" s="7" t="n">
-        <v>22.9</v>
-      </c>
-      <c r="L6" s="7" t="n">
-        <v>16.3</v>
-      </c>
-      <c r="M6" s="7" t="n">
-        <v>34</v>
-      </c>
-      <c r="N6" s="7" t="n">
-        <v>22</v>
-      </c>
       <c r="O6" s="7" t="n">
-        <v>292</v>
+        <v>264</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>41.67</v>
+        <v>43.58</v>
       </c>
       <c r="Q6" s="9" t="n">
-        <v>86.70999999999999</v>
+        <v>93.08</v>
       </c>
       <c r="R6" s="7" t="inlineStr">
         <is>
@@ -1255,7 +1253,7 @@
       </c>
       <c r="S6" s="10" t="inlineStr">
         <is>
-          <t>1 of the 75 listings this campaign advertises is out of stock (0 units). Ads are paused so spend does not keep running on items that cannot be bought.</t>
+          <t>1 of the 38 listings this campaign advertises is out of stock (0 units). Ads are paused so spend does not keep running on items that cannot be bought.</t>
         </is>
       </c>
       <c r="T6" s="7" t="inlineStr">
@@ -1268,12 +1266,12 @@
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>JD | Wall lights | New | Manual</t>
+          <t>JD | Ceiling Lights | Manual</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>164195009012</t>
+          <t>163193938012</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
@@ -1287,7 +1285,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>88</v>
+        <v>73</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>1</v>
@@ -1296,7 +1294,7 @@
         <v>0</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="I7" s="8" t="inlineStr">
         <is>
@@ -1309,25 +1307,25 @@
         </is>
       </c>
       <c r="K7" s="7" t="n">
-        <v>18.9</v>
+        <v>22</v>
       </c>
       <c r="L7" s="7" t="n">
-        <v>19</v>
+        <v>19.8</v>
       </c>
       <c r="M7" s="7" t="n">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="N7" s="7" t="n">
         <v>22</v>
       </c>
       <c r="O7" s="7" t="n">
-        <v>270</v>
+        <v>317</v>
       </c>
       <c r="P7" s="9" t="n">
-        <v>42</v>
+        <v>43.84</v>
       </c>
       <c r="Q7" s="9" t="n">
-        <v>81.8</v>
+        <v>86.63</v>
       </c>
       <c r="R7" s="7" t="inlineStr">
         <is>
@@ -1336,7 +1334,7 @@
       </c>
       <c r="S7" s="10" t="inlineStr">
         <is>
-          <t>1 of the 88 listings this campaign advertises is out of stock (0 units). Ads are paused so spend does not keep running on items that cannot be bought.</t>
+          <t>1 of the 73 listings this campaign advertises is out of stock (0 units). Ads are paused so spend does not keep running on items that cannot be bought.</t>
         </is>
       </c>
       <c r="T7" s="7" t="inlineStr">
@@ -1349,12 +1347,12 @@
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>JD | Spider Light | Manual</t>
+          <t>JD | Wall lights | New | Manual</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>17109990012</t>
+          <t>164195009012</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
@@ -1368,16 +1366,16 @@
         </is>
       </c>
       <c r="E8" s="7" t="n">
-        <v>16</v>
+        <v>80</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G8" s="7" t="n">
         <v>0</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I8" s="8" t="inlineStr">
         <is>
@@ -1390,25 +1388,25 @@
         </is>
       </c>
       <c r="K8" s="7" t="n">
-        <v>25.2</v>
+        <v>18.5</v>
       </c>
       <c r="L8" s="7" t="n">
-        <v>25</v>
+        <v>58.5</v>
       </c>
       <c r="M8" s="7" t="n">
-        <v>7</v>
+        <v>31</v>
       </c>
       <c r="N8" s="7" t="n">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="O8" s="7" t="n">
-        <v>196</v>
+        <v>270</v>
       </c>
       <c r="P8" s="9" t="n">
-        <v>36.7</v>
+        <v>42.42</v>
       </c>
       <c r="Q8" s="9" t="n">
-        <v>80.18000000000001</v>
+        <v>81.67</v>
       </c>
       <c r="R8" s="7" t="inlineStr">
         <is>
@@ -1417,7 +1415,7 @@
       </c>
       <c r="S8" s="10" t="inlineStr">
         <is>
-          <t>2 of the 16 listings this campaign advertises are out of stock (0 units). Ads are paused so spend does not keep running on items that cannot be bought.</t>
+          <t>1 of the 80 listings this campaign advertises is out of stock (0 units). Ads are paused so spend does not keep running on items that cannot be bought.</t>
         </is>
       </c>
       <c r="T8" s="7" t="inlineStr">
@@ -1430,12 +1428,12 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>JD | Mixed Product | Manual</t>
+          <t>JD | Spider Light | Manual</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>85734687012</t>
+          <t>17109990012</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
@@ -1449,10 +1447,10 @@
         </is>
       </c>
       <c r="E9" s="7" t="n">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G9" s="7" t="n">
         <v>0</v>
@@ -1460,34 +1458,34 @@
       <c r="H9" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="I9" s="11" t="inlineStr">
-        <is>
-          <t>Rule 1</t>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>Stock</t>
         </is>
       </c>
       <c r="J9" s="7" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="K9" s="7" t="n">
-        <v>55.8</v>
+        <v>25.6</v>
       </c>
       <c r="L9" s="7" t="n"/>
       <c r="M9" s="7" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="N9" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O9" s="7" t="n">
-        <v>210</v>
+        <v>199</v>
       </c>
       <c r="P9" s="9" t="n">
-        <v>35.49</v>
+        <v>37</v>
       </c>
       <c r="Q9" s="9" t="n">
-        <v>35.49</v>
+        <v>81.53</v>
       </c>
       <c r="R9" s="7" t="inlineStr">
         <is>
@@ -1496,7 +1494,7 @@
       </c>
       <c r="S9" s="10" t="inlineStr">
         <is>
-          <t>30-day ACOS is 55.8%, over the 40% ceiling. The last 7 days are showing no attributed sales at all — not below the 20% needed to count as an improving trend, so the campaign is paused.</t>
+          <t>2 of the 15 listings this campaign advertises are out of stock (0 units). Ads are paused so spend does not keep running on items that cannot be bought.</t>
         </is>
       </c>
       <c r="T9" s="7" t="inlineStr">
@@ -1509,332 +1507,328 @@
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
+          <t>JD | Target product | Manual</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>22831214012</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>RUNNING</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="n">
+        <v>44</v>
+      </c>
+      <c r="F10" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="11" t="inlineStr">
+        <is>
+          <t>Rule 1</t>
+        </is>
+      </c>
+      <c r="J10" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K10" s="7" t="n">
+        <v>48.6</v>
+      </c>
+      <c r="L10" s="7" t="n">
+        <v>50.3</v>
+      </c>
+      <c r="M10" s="7" t="n">
+        <v>17</v>
+      </c>
+      <c r="N10" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="O10" s="7" t="n">
+        <v>214</v>
+      </c>
+      <c r="P10" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="Q10" s="9" t="n">
+        <v>66.84999999999999</v>
+      </c>
+      <c r="R10" s="7" t="inlineStr">
+        <is>
+          <t>PAUSED</t>
+        </is>
+      </c>
+      <c r="S10" s="10" t="inlineStr">
+        <is>
+          <t>30-day ACOS is 48.6%, over the 40% ceiling. The last 7 days are still at 50.3% ACOS — not below the 20% needed to count as an improving trend, so the campaign is paused.</t>
+        </is>
+      </c>
+      <c r="T10" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="U10" s="7" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>JD | Mixed Product | Manual</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>85734687012</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>RUNNING</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="n">
+        <v>23</v>
+      </c>
+      <c r="F11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I11" s="11" t="inlineStr">
+        <is>
+          <t>Rule 1</t>
+        </is>
+      </c>
+      <c r="J11" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K11" s="7" t="n">
+        <v>79.90000000000001</v>
+      </c>
+      <c r="L11" s="7" t="n">
+        <v>71.59999999999999</v>
+      </c>
+      <c r="M11" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="N11" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="O11" s="7" t="n">
+        <v>270</v>
+      </c>
+      <c r="P11" s="9" t="n">
+        <v>44.32</v>
+      </c>
+      <c r="Q11" s="9" t="n">
+        <v>44.32</v>
+      </c>
+      <c r="R11" s="7" t="inlineStr">
+        <is>
+          <t>PAUSED</t>
+        </is>
+      </c>
+      <c r="S11" s="10" t="inlineStr">
+        <is>
+          <t>30-day ACOS is 79.9%, over the 40% ceiling. The last 7 days are still at 71.6% ACOS — not below the 20% needed to count as an improving trend, so the campaign is paused.</t>
+        </is>
+      </c>
+      <c r="T11" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="U11" s="7" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
           <t>JD | Steampunk | Theepana | Smart</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>165728546012</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C12" s="7" t="inlineStr">
         <is>
           <t>Smart</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
-        <is>
-          <t>RUNNING</t>
-        </is>
-      </c>
-      <c r="E10" s="7" t="n">
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>RUNNING</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="n">
         <v>20</v>
       </c>
-      <c r="F10" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" s="12" t="inlineStr">
+      <c r="F12" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="12" t="inlineStr">
         <is>
           <t>Rule 2</t>
         </is>
       </c>
-      <c r="J10" s="7" t="inlineStr">
+      <c r="J12" s="7" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="K10" s="7" t="n"/>
-      <c r="L10" s="7" t="n"/>
-      <c r="M10" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N10" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O10" s="7" t="n">
-        <v>90</v>
-      </c>
-      <c r="P10" s="9" t="n">
-        <v>18.16</v>
-      </c>
-      <c r="Q10" s="9" t="n">
-        <v>18.16</v>
-      </c>
-      <c r="R10" s="7" t="inlineStr">
+      <c r="K12" s="7" t="n"/>
+      <c r="L12" s="7" t="n"/>
+      <c r="M12" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="7" t="n">
+        <v>119</v>
+      </c>
+      <c r="P12" s="9" t="n">
+        <v>22.67</v>
+      </c>
+      <c r="Q12" s="9" t="n">
+        <v>22.67</v>
+      </c>
+      <c r="R12" s="7" t="inlineStr">
         <is>
           <t>PAUSED</t>
         </is>
       </c>
-      <c r="S10" s="10" t="inlineStr">
-        <is>
-          <t>90 clicks over 14 days produced zero orders, and spend of £18.16 is at or above the £2.50 floor — no longer cheap enough to justify keeping it live for the organic-ranking signal.</t>
-        </is>
-      </c>
-      <c r="T10" s="7" t="inlineStr">
+      <c r="S12" s="10" t="inlineStr">
+        <is>
+          <t>119 clicks over 14 days produced zero orders, and spend of £22.67 is at or above the £2.50 floor — no longer cheap enough to justify keeping it live for the organic-ranking signal.</t>
+        </is>
+      </c>
+      <c r="T12" s="7" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="U10" s="7" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="13" t="inlineStr">
-        <is>
-          <t>JD | PH |  All type | Transformer | Manual</t>
-        </is>
-      </c>
-      <c r="B11" s="13" t="inlineStr">
-        <is>
-          <t>129690774012</t>
-        </is>
-      </c>
-      <c r="C11" s="13" t="inlineStr">
+      <c r="U12" s="7" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>AH |Wall Lamp| manual</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>165722198012</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
         <is>
           <t>Manual</t>
         </is>
       </c>
-      <c r="D11" s="13" t="inlineStr">
-        <is>
-          <t>RUNNING</t>
-        </is>
-      </c>
-      <c r="E11" s="13" t="n">
-        <v>63</v>
-      </c>
-      <c r="F11" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="I11" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J11" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K11" s="13" t="n">
-        <v>32.6</v>
-      </c>
-      <c r="L11" s="13" t="n">
-        <v>20.7</v>
-      </c>
-      <c r="M11" s="13" t="n">
-        <v>27</v>
-      </c>
-      <c r="N11" s="13" t="n">
-        <v>15</v>
-      </c>
-      <c r="O11" s="13" t="n">
-        <v>342</v>
-      </c>
-      <c r="P11" s="14" t="n">
-        <v>67.52</v>
-      </c>
-      <c r="Q11" s="14" t="n">
-        <v>117.99</v>
-      </c>
-      <c r="R11" s="13" t="inlineStr">
-        <is>
-          <t>RUNNING</t>
-        </is>
-      </c>
-      <c r="S11" s="15" t="inlineStr">
-        <is>
-          <t>No rule matched — the campaign keeps running.</t>
-        </is>
-      </c>
-      <c r="T11" s="13" t="inlineStr">
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>RUNNING</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="F13" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="12" t="inlineStr">
+        <is>
+          <t>Rule 2</t>
+        </is>
+      </c>
+      <c r="J13" s="7" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="K13" s="7" t="n"/>
+      <c r="L13" s="7" t="n"/>
+      <c r="M13" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" s="7" t="n">
+        <v>34</v>
+      </c>
+      <c r="P13" s="9" t="n">
+        <v>6.44</v>
+      </c>
+      <c r="Q13" s="9" t="n">
+        <v>6.44</v>
+      </c>
+      <c r="R13" s="7" t="inlineStr">
+        <is>
+          <t>PAUSED</t>
+        </is>
+      </c>
+      <c r="S13" s="10" t="inlineStr">
+        <is>
+          <t>34 clicks over 14 days produced zero orders, and spend of £6.44 is at or above the £2.50 floor — no longer cheap enough to justify keeping it live for the organic-ranking signal.</t>
+        </is>
+      </c>
+      <c r="T13" s="7" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="U11" s="13" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="13" t="inlineStr">
-        <is>
-          <t>JD | PH | Tharsika | Lamp Holders | Manual</t>
-        </is>
-      </c>
-      <c r="B12" s="13" t="inlineStr">
-        <is>
-          <t>14841895012</t>
-        </is>
-      </c>
-      <c r="C12" s="13" t="inlineStr">
-        <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="D12" s="13" t="inlineStr">
-        <is>
-          <t>RUNNING</t>
-        </is>
-      </c>
-      <c r="E12" s="13" t="n">
-        <v>54</v>
-      </c>
-      <c r="F12" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="H12" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J12" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K12" s="13" t="n">
-        <v>30.3</v>
-      </c>
-      <c r="L12" s="13" t="n">
-        <v>40.1</v>
-      </c>
-      <c r="M12" s="13" t="n">
-        <v>58</v>
-      </c>
-      <c r="N12" s="13" t="n">
-        <v>32</v>
-      </c>
-      <c r="O12" s="13" t="n">
-        <v>363</v>
-      </c>
-      <c r="P12" s="14" t="n">
-        <v>52.92</v>
-      </c>
-      <c r="Q12" s="14" t="n">
-        <v>113.94</v>
-      </c>
-      <c r="R12" s="13" t="inlineStr">
-        <is>
-          <t>RUNNING</t>
-        </is>
-      </c>
-      <c r="S12" s="15" t="inlineStr">
-        <is>
-          <t>No rule matched — the campaign keeps running.</t>
-        </is>
-      </c>
-      <c r="T12" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="U12" s="13" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="13" t="inlineStr">
-        <is>
-          <t>JD | PH | BULB | TUWA | MANUAL</t>
-        </is>
-      </c>
-      <c r="B13" s="13" t="inlineStr">
-        <is>
-          <t>155338191012</t>
-        </is>
-      </c>
-      <c r="C13" s="13" t="inlineStr">
-        <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="D13" s="13" t="inlineStr">
-        <is>
-          <t>RUNNING</t>
-        </is>
-      </c>
-      <c r="E13" s="13" t="n">
-        <v>63</v>
-      </c>
-      <c r="F13" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J13" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K13" s="13" t="n">
-        <v>25.6</v>
-      </c>
-      <c r="L13" s="13" t="n">
-        <v>17.1</v>
-      </c>
-      <c r="M13" s="13" t="n">
-        <v>45</v>
-      </c>
-      <c r="N13" s="13" t="n">
-        <v>21</v>
-      </c>
-      <c r="O13" s="13" t="n">
-        <v>237</v>
-      </c>
-      <c r="P13" s="14" t="n">
-        <v>51.02</v>
-      </c>
-      <c r="Q13" s="14" t="n">
-        <v>110.42</v>
-      </c>
-      <c r="R13" s="13" t="inlineStr">
-        <is>
-          <t>RUNNING</t>
-        </is>
-      </c>
-      <c r="S13" s="15" t="inlineStr">
-        <is>
-          <t>No rule matched — the campaign keeps running.</t>
-        </is>
-      </c>
-      <c r="T13" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="U13" s="13" t="inlineStr"/>
+      <c r="U13" s="7" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="13" t="inlineStr">
         <is>
-          <t>JD | PH | PSU 4 types | Transformer | Manual</t>
+          <t>JD | PH |  All type | Transformer | Manual</t>
         </is>
       </c>
       <c r="B14" s="13" t="inlineStr">
         <is>
-          <t>34199100012</t>
+          <t>129690774012</t>
         </is>
       </c>
       <c r="C14" s="13" t="inlineStr">
@@ -1848,7 +1842,7 @@
         </is>
       </c>
       <c r="E14" s="13" t="n">
-        <v>12</v>
+        <v>63</v>
       </c>
       <c r="F14" s="13" t="n">
         <v>0</v>
@@ -1857,7 +1851,7 @@
         <v>0</v>
       </c>
       <c r="H14" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I14" s="13" t="inlineStr">
         <is>
@@ -1870,25 +1864,25 @@
         </is>
       </c>
       <c r="K14" s="13" t="n">
-        <v>20.4</v>
+        <v>20.9</v>
       </c>
       <c r="L14" s="13" t="n">
-        <v>22.5</v>
+        <v>9.1</v>
       </c>
       <c r="M14" s="13" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="N14" s="13" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="O14" s="13" t="n">
-        <v>213</v>
+        <v>368</v>
       </c>
       <c r="P14" s="14" t="n">
-        <v>50.33</v>
+        <v>67.22</v>
       </c>
       <c r="Q14" s="14" t="n">
-        <v>110.12</v>
+        <v>117.94</v>
       </c>
       <c r="R14" s="13" t="inlineStr">
         <is>
@@ -1910,17 +1904,17 @@
     <row r="15">
       <c r="A15" s="13" t="inlineStr">
         <is>
-          <t>JD | PH | power supply (fast moving) | Transformer  | smart</t>
+          <t>JD | PH | PSU 4 types | Transformer | Manual</t>
         </is>
       </c>
       <c r="B15" s="13" t="inlineStr">
         <is>
-          <t>28863466012</t>
+          <t>34199100012</t>
         </is>
       </c>
       <c r="C15" s="13" t="inlineStr">
         <is>
-          <t>Smart</t>
+          <t>Manual</t>
         </is>
       </c>
       <c r="D15" s="13" t="inlineStr">
@@ -1929,7 +1923,7 @@
         </is>
       </c>
       <c r="E15" s="13" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F15" s="13" t="n">
         <v>0</v>
@@ -1938,7 +1932,7 @@
         <v>0</v>
       </c>
       <c r="H15" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I15" s="13" t="inlineStr">
         <is>
@@ -1951,25 +1945,25 @@
         </is>
       </c>
       <c r="K15" s="13" t="n">
-        <v>24.1</v>
+        <v>18.2</v>
       </c>
       <c r="L15" s="13" t="n">
-        <v>34.1</v>
+        <v>18.5</v>
       </c>
       <c r="M15" s="13" t="n">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="N15" s="13" t="n">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="O15" s="13" t="n">
-        <v>257</v>
+        <v>229</v>
       </c>
       <c r="P15" s="14" t="n">
-        <v>51.75</v>
+        <v>54.03</v>
       </c>
       <c r="Q15" s="14" t="n">
-        <v>107.5</v>
+        <v>109.97</v>
       </c>
       <c r="R15" s="13" t="inlineStr">
         <is>
@@ -1991,12 +1985,12 @@
     <row r="16">
       <c r="A16" s="13" t="inlineStr">
         <is>
-          <t>JD | MH | LEDSONE Cable | Manual</t>
+          <t>JD | PH | BULB | TUWA | MANUAL</t>
         </is>
       </c>
       <c r="B16" s="13" t="inlineStr">
         <is>
-          <t>13950665012</t>
+          <t>155338191012</t>
         </is>
       </c>
       <c r="C16" s="13" t="inlineStr">
@@ -2010,7 +2004,7 @@
         </is>
       </c>
       <c r="E16" s="13" t="n">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="F16" s="13" t="n">
         <v>0</v>
@@ -2032,25 +2026,25 @@
         </is>
       </c>
       <c r="K16" s="13" t="n">
-        <v>20.4</v>
+        <v>32</v>
       </c>
       <c r="L16" s="13" t="n">
-        <v>13.1</v>
+        <v>13.8</v>
       </c>
       <c r="M16" s="13" t="n">
-        <v>69</v>
+        <v>29</v>
       </c>
       <c r="N16" s="13" t="n">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="O16" s="13" t="n">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="P16" s="14" t="n">
-        <v>44.08</v>
+        <v>52.74</v>
       </c>
       <c r="Q16" s="14" t="n">
-        <v>93.45</v>
+        <v>109.46</v>
       </c>
       <c r="R16" s="13" t="inlineStr">
         <is>
@@ -2072,12 +2066,12 @@
     <row r="17">
       <c r="A17" s="13" t="inlineStr">
         <is>
-          <t>JD | Plug in light | Manual</t>
+          <t>JD | PH | Tharsika | Lamp Holders | Manual</t>
         </is>
       </c>
       <c r="B17" s="13" t="inlineStr">
         <is>
-          <t>164267739012</t>
+          <t>14841895012</t>
         </is>
       </c>
       <c r="C17" s="13" t="inlineStr">
@@ -2091,7 +2085,7 @@
         </is>
       </c>
       <c r="E17" s="13" t="n">
-        <v>37</v>
+        <v>53</v>
       </c>
       <c r="F17" s="13" t="n">
         <v>0</v>
@@ -2100,7 +2094,7 @@
         <v>0</v>
       </c>
       <c r="H17" s="13" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="I17" s="13" t="inlineStr">
         <is>
@@ -2113,25 +2107,25 @@
         </is>
       </c>
       <c r="K17" s="13" t="n">
-        <v>16.7</v>
+        <v>28.2</v>
       </c>
       <c r="L17" s="13" t="n">
-        <v>27.5</v>
+        <v>33.1</v>
       </c>
       <c r="M17" s="13" t="n">
-        <v>38</v>
+        <v>60</v>
       </c>
       <c r="N17" s="13" t="n">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="O17" s="13" t="n">
-        <v>316</v>
+        <v>307</v>
       </c>
       <c r="P17" s="14" t="n">
-        <v>41.74</v>
+        <v>43.82</v>
       </c>
       <c r="Q17" s="14" t="n">
-        <v>91.91</v>
+        <v>105.66</v>
       </c>
       <c r="R17" s="13" t="inlineStr">
         <is>
@@ -2153,17 +2147,17 @@
     <row r="18">
       <c r="A18" s="13" t="inlineStr">
         <is>
-          <t>JD | MH | Flush Light &amp; Lamp Shade | Shanthini | Manual</t>
+          <t>JD | PH | power supply (fast moving) | Transformer  | smart</t>
         </is>
       </c>
       <c r="B18" s="13" t="inlineStr">
         <is>
-          <t>159902435012</t>
+          <t>28863466012</t>
         </is>
       </c>
       <c r="C18" s="13" t="inlineStr">
         <is>
-          <t>Manual</t>
+          <t>Smart</t>
         </is>
       </c>
       <c r="D18" s="13" t="inlineStr">
@@ -2172,7 +2166,7 @@
         </is>
       </c>
       <c r="E18" s="13" t="n">
-        <v>41</v>
+        <v>17</v>
       </c>
       <c r="F18" s="13" t="n">
         <v>0</v>
@@ -2181,7 +2175,7 @@
         <v>0</v>
       </c>
       <c r="H18" s="13" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="I18" s="13" t="inlineStr">
         <is>
@@ -2194,25 +2188,25 @@
         </is>
       </c>
       <c r="K18" s="13" t="n">
-        <v>39</v>
+        <v>26.5</v>
       </c>
       <c r="L18" s="13" t="n">
-        <v>222.9</v>
+        <v>40</v>
       </c>
       <c r="M18" s="13" t="n">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="N18" s="13" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="O18" s="13" t="n">
-        <v>251</v>
+        <v>258</v>
       </c>
       <c r="P18" s="14" t="n">
-        <v>41.69</v>
+        <v>51.68</v>
       </c>
       <c r="Q18" s="14" t="n">
-        <v>90.98</v>
+        <v>105.19</v>
       </c>
       <c r="R18" s="13" t="inlineStr">
         <is>
@@ -2234,12 +2228,12 @@
     <row r="19">
       <c r="A19" s="13" t="inlineStr">
         <is>
-          <t>JD | Target Transformer | Manual</t>
+          <t>JD | MH | LEDSONE Cable | Manual</t>
         </is>
       </c>
       <c r="B19" s="13" t="inlineStr">
         <is>
-          <t>161245031012</t>
+          <t>13950665012</t>
         </is>
       </c>
       <c r="C19" s="13" t="inlineStr">
@@ -2253,7 +2247,7 @@
         </is>
       </c>
       <c r="E19" s="13" t="n">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="F19" s="13" t="n">
         <v>0</v>
@@ -2262,7 +2256,7 @@
         <v>0</v>
       </c>
       <c r="H19" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I19" s="13" t="inlineStr">
         <is>
@@ -2275,25 +2269,25 @@
         </is>
       </c>
       <c r="K19" s="13" t="n">
-        <v>13.7</v>
+        <v>22.1</v>
       </c>
       <c r="L19" s="13" t="n">
-        <v>17.2</v>
+        <v>36</v>
       </c>
       <c r="M19" s="13" t="n">
-        <v>53</v>
+        <v>63</v>
       </c>
       <c r="N19" s="13" t="n">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="O19" s="13" t="n">
-        <v>214</v>
+        <v>237</v>
       </c>
       <c r="P19" s="14" t="n">
-        <v>43.48</v>
+        <v>44.19</v>
       </c>
       <c r="Q19" s="14" t="n">
-        <v>89.16</v>
+        <v>94.65000000000001</v>
       </c>
       <c r="R19" s="13" t="inlineStr">
         <is>
@@ -2315,12 +2309,12 @@
     <row r="20">
       <c r="A20" s="13" t="inlineStr">
         <is>
-          <t>JD | Cables | Target | Manual</t>
+          <t>JD | Target Transformer | Manual</t>
         </is>
       </c>
       <c r="B20" s="13" t="inlineStr">
         <is>
-          <t>161244718012</t>
+          <t>161245031012</t>
         </is>
       </c>
       <c r="C20" s="13" t="inlineStr">
@@ -2334,7 +2328,7 @@
         </is>
       </c>
       <c r="E20" s="13" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F20" s="13" t="n">
         <v>0</v>
@@ -2343,7 +2337,7 @@
         <v>0</v>
       </c>
       <c r="H20" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I20" s="13" t="inlineStr">
         <is>
@@ -2356,25 +2350,25 @@
         </is>
       </c>
       <c r="K20" s="13" t="n">
-        <v>16.4</v>
+        <v>13.6</v>
       </c>
       <c r="L20" s="13" t="n">
-        <v>14.4</v>
+        <v>14.3</v>
       </c>
       <c r="M20" s="13" t="n">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="N20" s="13" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="O20" s="13" t="n">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="P20" s="14" t="n">
-        <v>40.74</v>
+        <v>47.02</v>
       </c>
       <c r="Q20" s="14" t="n">
-        <v>88.16</v>
+        <v>91.11</v>
       </c>
       <c r="R20" s="13" t="inlineStr">
         <is>
@@ -2396,12 +2390,12 @@
     <row r="21">
       <c r="A21" s="13" t="inlineStr">
         <is>
-          <t>JD | PH | PLA | Power Supply | Transformer | Manual</t>
+          <t>JD | Plug in light | Manual</t>
         </is>
       </c>
       <c r="B21" s="13" t="inlineStr">
         <is>
-          <t>15603840012</t>
+          <t>164267739012</t>
         </is>
       </c>
       <c r="C21" s="13" t="inlineStr">
@@ -2415,7 +2409,7 @@
         </is>
       </c>
       <c r="E21" s="13" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="F21" s="13" t="n">
         <v>0</v>
@@ -2424,7 +2418,7 @@
         <v>0</v>
       </c>
       <c r="H21" s="13" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I21" s="13" t="inlineStr">
         <is>
@@ -2437,25 +2431,25 @@
         </is>
       </c>
       <c r="K21" s="13" t="n">
-        <v>31.5</v>
+        <v>19.7</v>
       </c>
       <c r="L21" s="13" t="n">
-        <v>68.2</v>
+        <v>18.6</v>
       </c>
       <c r="M21" s="13" t="n">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="N21" s="13" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="O21" s="13" t="n">
-        <v>183</v>
+        <v>318</v>
       </c>
       <c r="P21" s="14" t="n">
-        <v>44.22</v>
+        <v>42.97</v>
       </c>
       <c r="Q21" s="14" t="n">
-        <v>85.83</v>
+        <v>90.73999999999999</v>
       </c>
       <c r="R21" s="13" t="inlineStr">
         <is>
@@ -2477,12 +2471,12 @@
     <row r="22">
       <c r="A22" s="13" t="inlineStr">
         <is>
-          <t>JD | Without general | Manual</t>
+          <t>JD | PH | Pendant - II | Manual</t>
         </is>
       </c>
       <c r="B22" s="13" t="inlineStr">
         <is>
-          <t>144201913012</t>
+          <t>162961217012</t>
         </is>
       </c>
       <c r="C22" s="13" t="inlineStr">
@@ -2496,16 +2490,16 @@
         </is>
       </c>
       <c r="E22" s="13" t="n">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="F22" s="13" t="n">
         <v>0</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H22" s="13" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I22" s="13" t="inlineStr">
         <is>
@@ -2518,25 +2512,25 @@
         </is>
       </c>
       <c r="K22" s="13" t="n">
-        <v>31</v>
+        <v>21.8</v>
       </c>
       <c r="L22" s="13" t="n">
-        <v>28.7</v>
+        <v>12</v>
       </c>
       <c r="M22" s="13" t="n">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="N22" s="13" t="n">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="O22" s="13" t="n">
-        <v>230</v>
+        <v>292</v>
       </c>
       <c r="P22" s="14" t="n">
-        <v>51.93</v>
+        <v>42.83</v>
       </c>
       <c r="Q22" s="14" t="n">
-        <v>85.26000000000001</v>
+        <v>89.37</v>
       </c>
       <c r="R22" s="13" t="inlineStr">
         <is>
@@ -2558,12 +2552,12 @@
     <row r="23">
       <c r="A23" s="13" t="inlineStr">
         <is>
-          <t>JD | LJ | Lighting Parts | Thojika | Manual</t>
+          <t>JD | Without general | Manual</t>
         </is>
       </c>
       <c r="B23" s="13" t="inlineStr">
         <is>
-          <t>161735955012</t>
+          <t>144201913012</t>
         </is>
       </c>
       <c r="C23" s="13" t="inlineStr">
@@ -2577,13 +2571,13 @@
         </is>
       </c>
       <c r="E23" s="13" t="n">
-        <v>34</v>
+        <v>20</v>
       </c>
       <c r="F23" s="13" t="n">
         <v>0</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H23" s="13" t="n">
         <v>0</v>
@@ -2599,25 +2593,25 @@
         </is>
       </c>
       <c r="K23" s="13" t="n">
-        <v>32.7</v>
+        <v>24.7</v>
       </c>
       <c r="L23" s="13" t="n">
-        <v>14.5</v>
+        <v>13.8</v>
       </c>
       <c r="M23" s="13" t="n">
-        <v>25</v>
+        <v>52</v>
       </c>
       <c r="N23" s="13" t="n">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="O23" s="13" t="n">
-        <v>284</v>
+        <v>225</v>
       </c>
       <c r="P23" s="14" t="n">
-        <v>41.67</v>
+        <v>50.63</v>
       </c>
       <c r="Q23" s="14" t="n">
-        <v>84.47</v>
+        <v>87.73999999999999</v>
       </c>
       <c r="R23" s="13" t="inlineStr">
         <is>
@@ -2639,12 +2633,12 @@
     <row r="24">
       <c r="A24" s="13" t="inlineStr">
         <is>
-          <t>JD | PH | Pendant - II | Manual</t>
+          <t>JD | Cables | Target | Manual</t>
         </is>
       </c>
       <c r="B24" s="13" t="inlineStr">
         <is>
-          <t>162961217012</t>
+          <t>161244718012</t>
         </is>
       </c>
       <c r="C24" s="13" t="inlineStr">
@@ -2658,16 +2652,16 @@
         </is>
       </c>
       <c r="E24" s="13" t="n">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="F24" s="13" t="n">
         <v>0</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H24" s="13" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="I24" s="13" t="inlineStr">
         <is>
@@ -2680,25 +2674,25 @@
         </is>
       </c>
       <c r="K24" s="13" t="n">
-        <v>19.3</v>
+        <v>16.3</v>
       </c>
       <c r="L24" s="13" t="n">
-        <v>16.1</v>
+        <v>11.2</v>
       </c>
       <c r="M24" s="13" t="n">
-        <v>29</v>
+        <v>59</v>
       </c>
       <c r="N24" s="13" t="n">
-        <v>11</v>
+        <v>35</v>
       </c>
       <c r="O24" s="13" t="n">
-        <v>269</v>
+        <v>230</v>
       </c>
       <c r="P24" s="14" t="n">
-        <v>48.7</v>
+        <v>41.99</v>
       </c>
       <c r="Q24" s="14" t="n">
-        <v>84.25</v>
+        <v>86.31</v>
       </c>
       <c r="R24" s="13" t="inlineStr">
         <is>
@@ -2720,17 +2714,17 @@
     <row r="25">
       <c r="A25" s="13" t="inlineStr">
         <is>
-          <t>JD | Sm wall | smart</t>
+          <t>JD | PH | PLA | Power Supply | Transformer | Manual</t>
         </is>
       </c>
       <c r="B25" s="13" t="inlineStr">
         <is>
-          <t>17371404012</t>
+          <t>15603840012</t>
         </is>
       </c>
       <c r="C25" s="13" t="inlineStr">
         <is>
-          <t>Smart</t>
+          <t>Manual</t>
         </is>
       </c>
       <c r="D25" s="13" t="inlineStr">
@@ -2739,7 +2733,7 @@
         </is>
       </c>
       <c r="E25" s="13" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F25" s="13" t="n">
         <v>0</v>
@@ -2761,25 +2755,25 @@
         </is>
       </c>
       <c r="K25" s="13" t="n">
-        <v>19.7</v>
+        <v>34.8</v>
       </c>
       <c r="L25" s="13" t="n">
-        <v>14.4</v>
+        <v>152.2</v>
       </c>
       <c r="M25" s="13" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="N25" s="13" t="n">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="O25" s="13" t="n">
-        <v>307</v>
+        <v>209</v>
       </c>
       <c r="P25" s="14" t="n">
-        <v>49.03</v>
+        <v>47.68</v>
       </c>
       <c r="Q25" s="14" t="n">
-        <v>80.44</v>
+        <v>85.06999999999999</v>
       </c>
       <c r="R25" s="13" t="inlineStr">
         <is>
@@ -2801,17 +2795,17 @@
     <row r="26">
       <c r="A26" s="13" t="inlineStr">
         <is>
-          <t>JD | PLA | Light Product | Smart</t>
+          <t>JD | LJ | Lighting Parts | Thojika | Manual</t>
         </is>
       </c>
       <c r="B26" s="13" t="inlineStr">
         <is>
-          <t>15405904012</t>
+          <t>161735955012</t>
         </is>
       </c>
       <c r="C26" s="13" t="inlineStr">
         <is>
-          <t>Smart</t>
+          <t>Manual</t>
         </is>
       </c>
       <c r="D26" s="13" t="inlineStr">
@@ -2820,7 +2814,7 @@
         </is>
       </c>
       <c r="E26" s="13" t="n">
-        <v>14</v>
+        <v>33</v>
       </c>
       <c r="F26" s="13" t="n">
         <v>0</v>
@@ -2842,25 +2836,25 @@
         </is>
       </c>
       <c r="K26" s="13" t="n">
-        <v>15.8</v>
+        <v>32.6</v>
       </c>
       <c r="L26" s="13" t="n">
-        <v>24.1</v>
+        <v>19</v>
       </c>
       <c r="M26" s="13" t="n">
-        <v>46</v>
+        <v>25</v>
       </c>
       <c r="N26" s="13" t="n">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="O26" s="13" t="n">
-        <v>252</v>
+        <v>300</v>
       </c>
       <c r="P26" s="14" t="n">
-        <v>42.72</v>
+        <v>44.28</v>
       </c>
       <c r="Q26" s="14" t="n">
-        <v>80.09999999999999</v>
+        <v>84.62</v>
       </c>
       <c r="R26" s="13" t="inlineStr">
         <is>
@@ -2882,17 +2876,17 @@
     <row r="27">
       <c r="A27" s="13" t="inlineStr">
         <is>
-          <t>JD | PSU+Bulbs | Transformer | Manual</t>
+          <t>JD | Sm wall | smart</t>
         </is>
       </c>
       <c r="B27" s="13" t="inlineStr">
         <is>
-          <t>153333633012</t>
+          <t>17371404012</t>
         </is>
       </c>
       <c r="C27" s="13" t="inlineStr">
         <is>
-          <t>Manual</t>
+          <t>Smart</t>
         </is>
       </c>
       <c r="D27" s="13" t="inlineStr">
@@ -2901,7 +2895,7 @@
         </is>
       </c>
       <c r="E27" s="13" t="n">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="F27" s="13" t="n">
         <v>0</v>
@@ -2923,25 +2917,25 @@
         </is>
       </c>
       <c r="K27" s="13" t="n">
-        <v>30.8</v>
+        <v>19.3</v>
       </c>
       <c r="L27" s="13" t="n">
-        <v>22.8</v>
+        <v>46.8</v>
       </c>
       <c r="M27" s="13" t="n">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="N27" s="13" t="n">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="O27" s="13" t="n">
-        <v>197</v>
+        <v>284</v>
       </c>
       <c r="P27" s="14" t="n">
-        <v>44.58</v>
+        <v>46.13</v>
       </c>
       <c r="Q27" s="14" t="n">
-        <v>75.41</v>
+        <v>82.52</v>
       </c>
       <c r="R27" s="13" t="inlineStr">
         <is>
@@ -2963,172 +2957,174 @@
     <row r="28">
       <c r="A28" s="13" t="inlineStr">
         <is>
-          <t>JD | MH | Wall lights | Shimee | Manual</t>
+          <t>JD | PLA | Light Product | Smart</t>
         </is>
       </c>
       <c r="B28" s="13" t="inlineStr">
         <is>
-          <t>38338866012</t>
+          <t>15405904012</t>
         </is>
       </c>
       <c r="C28" s="13" t="inlineStr">
         <is>
+          <t>Smart</t>
+        </is>
+      </c>
+      <c r="D28" s="13" t="inlineStr">
+        <is>
+          <t>RUNNING</t>
+        </is>
+      </c>
+      <c r="E28" s="13" t="n">
+        <v>14</v>
+      </c>
+      <c r="F28" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J28" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K28" s="13" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="L28" s="13" t="n">
+        <v>31.3</v>
+      </c>
+      <c r="M28" s="13" t="n">
+        <v>41</v>
+      </c>
+      <c r="N28" s="13" t="n">
+        <v>26</v>
+      </c>
+      <c r="O28" s="13" t="n">
+        <v>263</v>
+      </c>
+      <c r="P28" s="14" t="n">
+        <v>44.08</v>
+      </c>
+      <c r="Q28" s="14" t="n">
+        <v>79.93000000000001</v>
+      </c>
+      <c r="R28" s="13" t="inlineStr">
+        <is>
+          <t>RUNNING</t>
+        </is>
+      </c>
+      <c r="S28" s="15" t="inlineStr">
+        <is>
+          <t>No rule matched — the campaign keeps running.</t>
+        </is>
+      </c>
+      <c r="T28" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="U28" s="13" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="13" t="inlineStr">
+        <is>
+          <t>JD | PSU+Bulbs | Transformer | Manual</t>
+        </is>
+      </c>
+      <c r="B29" s="13" t="inlineStr">
+        <is>
+          <t>153333633012</t>
+        </is>
+      </c>
+      <c r="C29" s="13" t="inlineStr">
+        <is>
           <t>Manual</t>
         </is>
       </c>
-      <c r="D28" s="13" t="inlineStr">
-        <is>
-          <t>RUNNING</t>
-        </is>
-      </c>
-      <c r="E28" s="13" t="n">
-        <v>8</v>
-      </c>
-      <c r="F28" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="G28" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="H28" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="I28" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J28" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K28" s="13" t="n">
-        <v>12.3</v>
-      </c>
-      <c r="L28" s="13" t="n">
-        <v>7.3</v>
-      </c>
-      <c r="M28" s="13" t="n">
-        <v>38</v>
-      </c>
-      <c r="N28" s="13" t="n">
-        <v>24</v>
-      </c>
-      <c r="O28" s="13" t="n">
-        <v>187</v>
-      </c>
-      <c r="P28" s="14" t="n">
-        <v>30.23</v>
-      </c>
-      <c r="Q28" s="14" t="n">
-        <v>66.36</v>
-      </c>
-      <c r="R28" s="13" t="inlineStr">
-        <is>
-          <t>RUNNING</t>
-        </is>
-      </c>
-      <c r="S28" s="15" t="inlineStr">
+      <c r="D29" s="13" t="inlineStr">
+        <is>
+          <t>RUNNING</t>
+        </is>
+      </c>
+      <c r="E29" s="13" t="n">
+        <v>9</v>
+      </c>
+      <c r="F29" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J29" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K29" s="13" t="n">
+        <v>30.2</v>
+      </c>
+      <c r="L29" s="13" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="M29" s="13" t="n">
+        <v>35</v>
+      </c>
+      <c r="N29" s="13" t="n">
+        <v>25</v>
+      </c>
+      <c r="O29" s="13" t="n">
+        <v>220</v>
+      </c>
+      <c r="P29" s="14" t="n">
+        <v>49.5</v>
+      </c>
+      <c r="Q29" s="14" t="n">
+        <v>79.38</v>
+      </c>
+      <c r="R29" s="13" t="inlineStr">
+        <is>
+          <t>RUNNING</t>
+        </is>
+      </c>
+      <c r="S29" s="15" t="inlineStr">
         <is>
           <t>No rule matched — the campaign keeps running.</t>
         </is>
       </c>
-      <c r="T28" s="13" t="inlineStr">
+      <c r="T29" s="13" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="U28" s="13" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="16" t="inlineStr">
-        <is>
-          <t>JD | PH | Abinayaa | Light Fittings | Manual</t>
-        </is>
-      </c>
-      <c r="B29" s="16" t="inlineStr">
-        <is>
-          <t>155945896012</t>
-        </is>
-      </c>
-      <c r="C29" s="16" t="inlineStr">
-        <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="D29" s="16" t="inlineStr">
-        <is>
-          <t>ENDED</t>
-        </is>
-      </c>
-      <c r="E29" s="16" t="n">
-        <v>39</v>
-      </c>
-      <c r="F29" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="G29" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="H29" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="I29" s="16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J29" s="16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K29" s="16" t="n">
-        <v>31.8</v>
-      </c>
-      <c r="L29" s="16" t="n"/>
-      <c r="M29" s="16" t="n">
-        <v>23</v>
-      </c>
-      <c r="N29" s="16" t="n">
-        <v>3</v>
-      </c>
-      <c r="O29" s="16" t="n">
-        <v>130</v>
-      </c>
-      <c r="P29" s="17" t="n">
-        <v>26.34</v>
-      </c>
-      <c r="Q29" s="17" t="n">
-        <v>66.18000000000001</v>
-      </c>
-      <c r="R29" s="16" t="inlineStr">
-        <is>
-          <t>ALREADY OFF</t>
-        </is>
-      </c>
-      <c r="S29" s="18" t="inlineStr">
-        <is>
-          <t>Campaign is already ENDED. No pause action taken — the rules are not evaluated against a campaign that is not running.</t>
-        </is>
-      </c>
-      <c r="T29" s="16" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="U29" s="16" t="inlineStr"/>
+      <c r="U29" s="13" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="13" t="inlineStr">
         <is>
-          <t>JD | PH | Flush light | Manual</t>
+          <t>JD | MH | Wall lights | Shimee | Manual</t>
         </is>
       </c>
       <c r="B30" s="13" t="inlineStr">
         <is>
-          <t>26896653012</t>
+          <t>38338866012</t>
         </is>
       </c>
       <c r="C30" s="13" t="inlineStr">
@@ -3142,7 +3138,7 @@
         </is>
       </c>
       <c r="E30" s="13" t="n">
-        <v>36</v>
+        <v>7</v>
       </c>
       <c r="F30" s="13" t="n">
         <v>0</v>
@@ -3151,7 +3147,7 @@
         <v>0</v>
       </c>
       <c r="H30" s="13" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I30" s="13" t="inlineStr">
         <is>
@@ -3164,25 +3160,25 @@
         </is>
       </c>
       <c r="K30" s="13" t="n">
-        <v>20.3</v>
+        <v>11.2</v>
       </c>
       <c r="L30" s="13" t="n">
-        <v>13.4</v>
+        <v>6.2</v>
       </c>
       <c r="M30" s="13" t="n">
-        <v>27</v>
+        <v>41</v>
       </c>
       <c r="N30" s="13" t="n">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="O30" s="13" t="n">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="P30" s="14" t="n">
-        <v>27.12</v>
+        <v>26.79</v>
       </c>
       <c r="Q30" s="14" t="n">
-        <v>64.48</v>
+        <v>65.97</v>
       </c>
       <c r="R30" s="13" t="inlineStr">
         <is>
@@ -3204,12 +3200,12 @@
     <row r="31">
       <c r="A31" s="13" t="inlineStr">
         <is>
-          <t>JD | Target product | Manual</t>
+          <t>JD | Cables | Video | Manual</t>
         </is>
       </c>
       <c r="B31" s="13" t="inlineStr">
         <is>
-          <t>22831214012</t>
+          <t>165065723012</t>
         </is>
       </c>
       <c r="C31" s="13" t="inlineStr">
@@ -3223,47 +3219,47 @@
         </is>
       </c>
       <c r="E31" s="13" t="n">
+        <v>8</v>
+      </c>
+      <c r="F31" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J31" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K31" s="13" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="L31" s="13" t="n">
+        <v>25.6</v>
+      </c>
+      <c r="M31" s="13" t="n">
         <v>44</v>
       </c>
-      <c r="F31" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="G31" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="H31" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="I31" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J31" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K31" s="13" t="n">
-        <v>37.7</v>
-      </c>
-      <c r="L31" s="13" t="n">
-        <v>35.4</v>
-      </c>
-      <c r="M31" s="13" t="n">
-        <v>21</v>
-      </c>
       <c r="N31" s="13" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="O31" s="13" t="n">
-        <v>226</v>
+        <v>202</v>
       </c>
       <c r="P31" s="14" t="n">
-        <v>43.85</v>
+        <v>38.54</v>
       </c>
       <c r="Q31" s="14" t="n">
-        <v>64.09</v>
+        <v>65.61</v>
       </c>
       <c r="R31" s="13" t="inlineStr">
         <is>
@@ -3283,93 +3279,95 @@
       <c r="U31" s="13" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="16" t="inlineStr">
-        <is>
-          <t>JD | MH | 3 head Pendent | Smart</t>
-        </is>
-      </c>
-      <c r="B32" s="16" t="inlineStr">
-        <is>
-          <t>135730419012</t>
-        </is>
-      </c>
-      <c r="C32" s="16" t="inlineStr">
-        <is>
-          <t>Smart</t>
-        </is>
-      </c>
-      <c r="D32" s="16" t="inlineStr">
-        <is>
-          <t>ENDED</t>
-        </is>
-      </c>
-      <c r="E32" s="16" t="n">
-        <v>28</v>
-      </c>
-      <c r="F32" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="G32" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="H32" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="I32" s="16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J32" s="16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K32" s="16" t="n">
-        <v>26.1</v>
-      </c>
-      <c r="L32" s="16" t="n"/>
-      <c r="M32" s="16" t="n">
-        <v>5</v>
-      </c>
-      <c r="N32" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="O32" s="16" t="n">
-        <v>97</v>
-      </c>
-      <c r="P32" s="17" t="n">
-        <v>24.09</v>
-      </c>
-      <c r="Q32" s="17" t="n">
-        <v>62.98</v>
-      </c>
-      <c r="R32" s="16" t="inlineStr">
-        <is>
-          <t>ALREADY OFF</t>
-        </is>
-      </c>
-      <c r="S32" s="18" t="inlineStr">
-        <is>
-          <t>Campaign is already ENDED. No pause action taken — the rules are not evaluated against a campaign that is not running.</t>
-        </is>
-      </c>
-      <c r="T32" s="16" t="inlineStr">
+      <c r="A32" s="13" t="inlineStr">
+        <is>
+          <t>JD | PH | Flush light | Manual</t>
+        </is>
+      </c>
+      <c r="B32" s="13" t="inlineStr">
+        <is>
+          <t>26896653012</t>
+        </is>
+      </c>
+      <c r="C32" s="13" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="D32" s="13" t="inlineStr">
+        <is>
+          <t>RUNNING</t>
+        </is>
+      </c>
+      <c r="E32" s="13" t="n">
+        <v>36</v>
+      </c>
+      <c r="F32" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="I32" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J32" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K32" s="13" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="L32" s="13" t="n">
+        <v>14</v>
+      </c>
+      <c r="M32" s="13" t="n">
+        <v>26</v>
+      </c>
+      <c r="N32" s="13" t="n">
+        <v>16</v>
+      </c>
+      <c r="O32" s="13" t="n">
+        <v>157</v>
+      </c>
+      <c r="P32" s="14" t="n">
+        <v>27.27</v>
+      </c>
+      <c r="Q32" s="14" t="n">
+        <v>62.4</v>
+      </c>
+      <c r="R32" s="13" t="inlineStr">
+        <is>
+          <t>RUNNING</t>
+        </is>
+      </c>
+      <c r="S32" s="15" t="inlineStr">
+        <is>
+          <t>No rule matched — the campaign keeps running.</t>
+        </is>
+      </c>
+      <c r="T32" s="13" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="U32" s="16" t="inlineStr"/>
+      <c r="U32" s="13" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="13" t="inlineStr">
         <is>
-          <t>JD | Cables | Video | Manual</t>
+          <t>JD | Wall light + video campaign</t>
         </is>
       </c>
       <c r="B33" s="13" t="inlineStr">
         <is>
-          <t>165065723012</t>
+          <t>163055118012</t>
         </is>
       </c>
       <c r="C33" s="13" t="inlineStr">
@@ -3383,7 +3381,7 @@
         </is>
       </c>
       <c r="E33" s="13" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="F33" s="13" t="n">
         <v>0</v>
@@ -3405,25 +3403,25 @@
         </is>
       </c>
       <c r="K33" s="13" t="n">
-        <v>18.1</v>
+        <v>18</v>
       </c>
       <c r="L33" s="13" t="n">
-        <v>20.7</v>
+        <v>38.8</v>
       </c>
       <c r="M33" s="13" t="n">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="N33" s="13" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="O33" s="13" t="n">
-        <v>183</v>
+        <v>197</v>
       </c>
       <c r="P33" s="14" t="n">
-        <v>34.4</v>
+        <v>36.89</v>
       </c>
       <c r="Q33" s="14" t="n">
-        <v>61.41</v>
+        <v>59.15</v>
       </c>
       <c r="R33" s="13" t="inlineStr">
         <is>
@@ -3443,100 +3441,98 @@
       <c r="U33" s="13" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="13" t="inlineStr">
-        <is>
-          <t>JD | Wall light + video campaign</t>
-        </is>
-      </c>
-      <c r="B34" s="13" t="inlineStr">
-        <is>
-          <t>163055118012</t>
-        </is>
-      </c>
-      <c r="C34" s="13" t="inlineStr">
-        <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="D34" s="13" t="inlineStr">
-        <is>
-          <t>RUNNING</t>
-        </is>
-      </c>
-      <c r="E34" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="F34" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="G34" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="H34" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="I34" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J34" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K34" s="13" t="n">
-        <v>19.3</v>
-      </c>
-      <c r="L34" s="13" t="n">
-        <v>10.8</v>
-      </c>
-      <c r="M34" s="13" t="n">
-        <v>21</v>
-      </c>
-      <c r="N34" s="13" t="n">
-        <v>17</v>
-      </c>
-      <c r="O34" s="13" t="n">
-        <v>199</v>
-      </c>
-      <c r="P34" s="14" t="n">
-        <v>35.81</v>
-      </c>
-      <c r="Q34" s="14" t="n">
-        <v>59.95</v>
-      </c>
-      <c r="R34" s="13" t="inlineStr">
-        <is>
-          <t>RUNNING</t>
-        </is>
-      </c>
-      <c r="S34" s="15" t="inlineStr">
-        <is>
-          <t>No rule matched — the campaign keeps running.</t>
-        </is>
-      </c>
-      <c r="T34" s="13" t="inlineStr">
+      <c r="A34" s="16" t="inlineStr">
+        <is>
+          <t>JD | MH | 3 head Pendent | Smart</t>
+        </is>
+      </c>
+      <c r="B34" s="16" t="inlineStr">
+        <is>
+          <t>135730419012</t>
+        </is>
+      </c>
+      <c r="C34" s="16" t="inlineStr">
+        <is>
+          <t>Smart</t>
+        </is>
+      </c>
+      <c r="D34" s="16" t="inlineStr">
+        <is>
+          <t>ENDED</t>
+        </is>
+      </c>
+      <c r="E34" s="16" t="n">
+        <v>28</v>
+      </c>
+      <c r="F34" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="H34" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J34" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K34" s="16" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="L34" s="16" t="n"/>
+      <c r="M34" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="N34" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="O34" s="16" t="n">
+        <v>73</v>
+      </c>
+      <c r="P34" s="17" t="n">
+        <v>18.32</v>
+      </c>
+      <c r="Q34" s="17" t="n">
+        <v>55.9</v>
+      </c>
+      <c r="R34" s="16" t="inlineStr">
+        <is>
+          <t>ALREADY OFF</t>
+        </is>
+      </c>
+      <c r="S34" s="18" t="inlineStr">
+        <is>
+          <t>Campaign is already ENDED. No pause action taken — the rules are not evaluated against a campaign that is not running.</t>
+        </is>
+      </c>
+      <c r="T34" s="16" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="U34" s="13" t="inlineStr"/>
+      <c r="U34" s="16" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="16" t="inlineStr">
         <is>
-          <t>JD | PLA | Pendent Lights | Smart</t>
+          <t>JD | PH | Abinayaa | Light Fittings | Manual</t>
         </is>
       </c>
       <c r="B35" s="16" t="inlineStr">
         <is>
-          <t>15405839012</t>
+          <t>155945896012</t>
         </is>
       </c>
       <c r="C35" s="16" t="inlineStr">
         <is>
-          <t>Smart</t>
+          <t>Manual</t>
         </is>
       </c>
       <c r="D35" s="16" t="inlineStr">
@@ -3545,10 +3541,10 @@
         </is>
       </c>
       <c r="E35" s="16" t="n">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F35" s="16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G35" s="16" t="n">
         <v>0</v>
@@ -3566,22 +3562,24 @@
           <t>—</t>
         </is>
       </c>
-      <c r="K35" s="16" t="n"/>
+      <c r="K35" s="16" t="n">
+        <v>31.9</v>
+      </c>
       <c r="L35" s="16" t="n"/>
       <c r="M35" s="16" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="N35" s="16" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O35" s="16" t="n">
-        <v>0</v>
+        <v>101</v>
       </c>
       <c r="P35" s="17" t="n">
-        <v>0</v>
+        <v>20.02</v>
       </c>
       <c r="Q35" s="17" t="n">
-        <v>37.65</v>
+        <v>55.79</v>
       </c>
       <c r="R35" s="16" t="inlineStr">
         <is>
@@ -3601,110 +3599,112 @@
       <c r="U35" s="16" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="16" t="inlineStr">
-        <is>
-          <t>JD | MH | Cables | Jasmini | Smart</t>
-        </is>
-      </c>
-      <c r="B36" s="16" t="inlineStr">
-        <is>
-          <t>28863417012</t>
-        </is>
-      </c>
-      <c r="C36" s="16" t="inlineStr">
-        <is>
-          <t>Smart</t>
-        </is>
-      </c>
-      <c r="D36" s="16" t="inlineStr">
-        <is>
-          <t>PAUSED</t>
-        </is>
-      </c>
-      <c r="E36" s="16" t="n">
-        <v>6</v>
-      </c>
-      <c r="F36" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="G36" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="H36" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="I36" s="16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J36" s="16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K36" s="16" t="n">
-        <v>46</v>
-      </c>
-      <c r="L36" s="16" t="n"/>
-      <c r="M36" s="16" t="n">
-        <v>13</v>
-      </c>
-      <c r="N36" s="16" t="n">
-        <v>2</v>
-      </c>
-      <c r="O36" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="P36" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q36" s="17" t="n">
-        <v>34.12</v>
-      </c>
-      <c r="R36" s="16" t="inlineStr">
-        <is>
-          <t>ALREADY OFF</t>
-        </is>
-      </c>
-      <c r="S36" s="18" t="inlineStr">
-        <is>
-          <t>Campaign is already PAUSED. No pause action taken — the rules are not evaluated against a campaign that is not running.</t>
-        </is>
-      </c>
-      <c r="T36" s="16" t="inlineStr">
+      <c r="A36" s="13" t="inlineStr">
+        <is>
+          <t>AH- 30/07/2026, 10:27</t>
+        </is>
+      </c>
+      <c r="B36" s="13" t="inlineStr">
+        <is>
+          <t>165612935012</t>
+        </is>
+      </c>
+      <c r="C36" s="13" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="D36" s="13" t="inlineStr">
+        <is>
+          <t>RUNNING</t>
+        </is>
+      </c>
+      <c r="E36" s="13" t="n">
+        <v>18</v>
+      </c>
+      <c r="F36" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I36" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J36" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K36" s="13" t="n">
+        <v>28.4</v>
+      </c>
+      <c r="L36" s="13" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="M36" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="N36" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="O36" s="13" t="n">
+        <v>177</v>
+      </c>
+      <c r="P36" s="14" t="n">
+        <v>35.02</v>
+      </c>
+      <c r="Q36" s="14" t="n">
+        <v>38.02</v>
+      </c>
+      <c r="R36" s="13" t="inlineStr">
+        <is>
+          <t>RUNNING</t>
+        </is>
+      </c>
+      <c r="S36" s="15" t="inlineStr">
+        <is>
+          <t>No rule matched — the campaign keeps running.</t>
+        </is>
+      </c>
+      <c r="T36" s="13" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="U36" s="16" t="inlineStr"/>
+      <c r="U36" s="13" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="16" t="inlineStr">
         <is>
-          <t>JD | PH | Lampshade  | Utharsika | Manual</t>
+          <t>JD | PLA | Pendent Lights | Smart</t>
         </is>
       </c>
       <c r="B37" s="16" t="inlineStr">
         <is>
-          <t>129690966012</t>
+          <t>15405839012</t>
         </is>
       </c>
       <c r="C37" s="16" t="inlineStr">
         <is>
-          <t>Manual</t>
+          <t>Smart</t>
         </is>
       </c>
       <c r="D37" s="16" t="inlineStr">
         <is>
-          <t>PAUSED</t>
+          <t>ENDED</t>
         </is>
       </c>
       <c r="E37" s="16" t="n">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="F37" s="16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G37" s="16" t="n">
         <v>0</v>
@@ -3722,26 +3722,22 @@
           <t>—</t>
         </is>
       </c>
-      <c r="K37" s="16" t="n">
-        <v>48.3</v>
-      </c>
-      <c r="L37" s="16" t="n">
-        <v>0</v>
-      </c>
+      <c r="K37" s="16" t="n"/>
+      <c r="L37" s="16" t="n"/>
       <c r="M37" s="16" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N37" s="16" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O37" s="16" t="n">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="P37" s="17" t="n">
-        <v>12.08</v>
+        <v>0</v>
       </c>
       <c r="Q37" s="17" t="n">
-        <v>30.78</v>
+        <v>26.19</v>
       </c>
       <c r="R37" s="16" t="inlineStr">
         <is>
@@ -3750,7 +3746,7 @@
       </c>
       <c r="S37" s="18" t="inlineStr">
         <is>
-          <t>Campaign is already PAUSED. No pause action taken — the rules are not evaluated against a campaign that is not running.</t>
+          <t>Campaign is already ENDED. No pause action taken — the rules are not evaluated against a campaign that is not running.</t>
         </is>
       </c>
       <c r="T37" s="16" t="inlineStr">
@@ -3763,12 +3759,12 @@
     <row r="38">
       <c r="A38" s="16" t="inlineStr">
         <is>
-          <t>AH- 30/07/2026, 10:27</t>
+          <t>JD | PH | Lampshade  | Utharsika | Manual</t>
         </is>
       </c>
       <c r="B38" s="16" t="inlineStr">
         <is>
-          <t>165612935012</t>
+          <t>129690966012</t>
         </is>
       </c>
       <c r="C38" s="16" t="inlineStr">
@@ -3782,7 +3778,7 @@
         </is>
       </c>
       <c r="E38" s="16" t="n">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="F38" s="16" t="n">
         <v>0</v>
@@ -3804,25 +3800,23 @@
         </is>
       </c>
       <c r="K38" s="16" t="n">
-        <v>59.9</v>
-      </c>
-      <c r="L38" s="16" t="n">
-        <v>40.6</v>
-      </c>
+        <v>37.7</v>
+      </c>
+      <c r="L38" s="16" t="n"/>
       <c r="M38" s="16" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="N38" s="16" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="O38" s="16" t="n">
-        <v>118</v>
+        <v>75</v>
       </c>
       <c r="P38" s="17" t="n">
-        <v>22.04</v>
+        <v>12.08</v>
       </c>
       <c r="Q38" s="17" t="n">
-        <v>22.04</v>
+        <v>24</v>
       </c>
       <c r="R38" s="16" t="inlineStr">
         <is>
@@ -3844,17 +3838,17 @@
     <row r="39">
       <c r="A39" s="16" t="inlineStr">
         <is>
-          <t>JD | MH | Hemp Lights | Renuha | Manual</t>
+          <t>JD | MH | Cables | Jasmini | Smart</t>
         </is>
       </c>
       <c r="B39" s="16" t="inlineStr">
         <is>
-          <t>155212621012</t>
+          <t>28863417012</t>
         </is>
       </c>
       <c r="C39" s="16" t="inlineStr">
         <is>
-          <t>Manual</t>
+          <t>Smart</t>
         </is>
       </c>
       <c r="D39" s="16" t="inlineStr">
@@ -3863,7 +3857,7 @@
         </is>
       </c>
       <c r="E39" s="16" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F39" s="16" t="n">
         <v>0</v>
@@ -3884,10 +3878,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="K39" s="16" t="n"/>
+      <c r="K39" s="16" t="n">
+        <v>51</v>
+      </c>
       <c r="L39" s="16" t="n"/>
       <c r="M39" s="16" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="N39" s="16" t="n">
         <v>0</v>
@@ -3899,7 +3895,7 @@
         <v>0</v>
       </c>
       <c r="Q39" s="17" t="n">
-        <v>20.16</v>
+        <v>21.28</v>
       </c>
       <c r="R39" s="16" t="inlineStr">
         <is>
@@ -3921,17 +3917,17 @@
     <row r="40">
       <c r="A40" s="16" t="inlineStr">
         <is>
-          <t>JD  | Shade+video campaign</t>
+          <t>JD | MH | Hemp Lights | Renuha | Manual</t>
         </is>
       </c>
       <c r="B40" s="16" t="inlineStr">
         <is>
-          <t>163710397012</t>
+          <t>155212621012</t>
         </is>
       </c>
       <c r="C40" s="16" t="inlineStr">
         <is>
-          <t>Smart</t>
+          <t>Manual</t>
         </is>
       </c>
       <c r="D40" s="16" t="inlineStr">
@@ -3940,7 +3936,7 @@
         </is>
       </c>
       <c r="E40" s="16" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F40" s="16" t="n">
         <v>0</v>
@@ -3949,7 +3945,7 @@
         <v>0</v>
       </c>
       <c r="H40" s="16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I40" s="16" t="inlineStr">
         <is>
@@ -3961,12 +3957,10 @@
           <t>—</t>
         </is>
       </c>
-      <c r="K40" s="16" t="n">
-        <v>93.7</v>
-      </c>
+      <c r="K40" s="16" t="n"/>
       <c r="L40" s="16" t="n"/>
       <c r="M40" s="16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N40" s="16" t="n">
         <v>0</v>
@@ -3978,7 +3972,7 @@
         <v>0</v>
       </c>
       <c r="Q40" s="17" t="n">
-        <v>9.359999999999999</v>
+        <v>11.33</v>
       </c>
       <c r="R40" s="16" t="inlineStr">
         <is>
@@ -4000,17 +3994,17 @@
     <row r="41">
       <c r="A41" s="16" t="inlineStr">
         <is>
-          <t>AH |Wall Lamp| manual</t>
+          <t>JD  | Shade+video campaign</t>
         </is>
       </c>
       <c r="B41" s="16" t="inlineStr">
         <is>
-          <t>165722198012</t>
+          <t>163710397012</t>
         </is>
       </c>
       <c r="C41" s="16" t="inlineStr">
         <is>
-          <t>Manual</t>
+          <t>Smart</t>
         </is>
       </c>
       <c r="D41" s="16" t="inlineStr">
@@ -4019,7 +4013,7 @@
         </is>
       </c>
       <c r="E41" s="16" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="F41" s="16" t="n">
         <v>0</v>
@@ -4028,7 +4022,7 @@
         <v>0</v>
       </c>
       <c r="H41" s="16" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I41" s="16" t="inlineStr">
         <is>
@@ -4040,22 +4034,24 @@
           <t>—</t>
         </is>
       </c>
-      <c r="K41" s="16" t="n"/>
+      <c r="K41" s="16" t="n">
+        <v>83.5</v>
+      </c>
       <c r="L41" s="16" t="n"/>
       <c r="M41" s="16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N41" s="16" t="n">
         <v>0</v>
       </c>
       <c r="O41" s="16" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="P41" s="17" t="n">
-        <v>1.68</v>
+        <v>0</v>
       </c>
       <c r="Q41" s="17" t="n">
-        <v>1.68</v>
+        <v>8.34</v>
       </c>
       <c r="R41" s="16" t="inlineStr">
         <is>
@@ -4840,7 +4836,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>12 Jul - 10 Aug 2026</t>
+          <t>15 Jul - 13 Aug 2026</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -4857,7 +4853,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>28 Jul - 10 Aug 2026</t>
+          <t>31 Jul - 13 Aug 2026</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -4874,7 +4870,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>4-10 Aug 2026</t>
+          <t>7-13 Aug 2026</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">

</xml_diff>